<commit_message>
poniendo foto solo de la curcuma en la data de productos, y cambiando el numero de whatsapp a mi numero real para que me lleguen los pedidos.
</commit_message>
<xml_diff>
--- a/pedidos_yuyos.xlsx
+++ b/pedidos_yuyos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -432,9 +432,64 @@
         <v>2500</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>15/9/2026, 08:01:04</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Cúrcuma en Raíz</v>
+      </c>
+      <c r="C4">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>15/9/2026, 08:02:08</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Cúrcuma en Raíz</v>
+      </c>
+      <c r="C5">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>15/9/2026, 08:02:31</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Cúrcuma en Raíz</v>
+      </c>
+      <c r="C6">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>15/9/2026, 08:02:48</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Cúrcuma en Raíz</v>
+      </c>
+      <c r="C7">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>15/9/2026, 08:03:24</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Cúrcuma en Raíz</v>
+      </c>
+      <c r="C8">
+        <v>2500</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>